<commit_message>
Move Kennedy's Nov night-float off the 11/1-6 flight week; drop green highlight
- Kennedy's November NF week moved to 11/15-20 so Fri 11/6 is a short call and
  he is off for the Nov 7-8 weekend (Friday night float rounds into Saturday AM).
- Remove the green shading on Kennedy's cells; LSH now use the standard color.
- Regenerate all monthly workbooks and the compliance report. Still 0 hard-rule
  violations; every LSH intern keeps exactly 1 NF week + 1 Saturday/month.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J6EM8SxuZs5C898HeFBgt7
</commit_message>
<xml_diff>
--- a/intern_schedule_2026-2027/schedules/TYP_Intern_Schedule_Oct2026-Jun2027.xlsx
+++ b/intern_schedule_2026-2027/schedules/TYP_Intern_Schedule_Oct2026-Jun2027.xlsx
@@ -45,7 +45,7 @@
       <i val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -67,11 +67,6 @@
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -91,7 +86,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -108,9 +103,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1476,9 +1468,9 @@
         </is>
       </c>
       <c r="D3" s="5" t="n"/>
-      <c r="E3" s="8" t="inlineStr">
-        <is>
-          <t>KENNEDY</t>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>WISE</t>
         </is>
       </c>
     </row>
@@ -1493,17 +1485,17 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
+          <t>KENNEDY</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>MULLINS, CHIASSON</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
           <t>WISE</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>MULLINS, CHIASSON</t>
-        </is>
-      </c>
-      <c r="E4" s="8" t="inlineStr">
-        <is>
-          <t>KENNEDY</t>
         </is>
       </c>
     </row>
@@ -1523,12 +1515,12 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>WISE, CHIASSON</t>
-        </is>
-      </c>
-      <c r="E5" s="8" t="inlineStr">
-        <is>
-          <t>KENNEDY</t>
+          <t>KENNEDY, CHIASSON</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>WISE</t>
         </is>
       </c>
     </row>
@@ -1548,12 +1540,12 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>WISE, MULLINS</t>
-        </is>
-      </c>
-      <c r="E6" s="8" t="inlineStr">
-        <is>
-          <t>KENNEDY</t>
+          <t>KENNEDY, MULLINS</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>WISE</t>
         </is>
       </c>
     </row>
@@ -1576,9 +1568,9 @@
           <t>CHIASSON</t>
         </is>
       </c>
-      <c r="E7" s="8" t="inlineStr">
-        <is>
-          <t>KENNEDY</t>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>WISE</t>
         </is>
       </c>
     </row>
@@ -1593,17 +1585,17 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
+          <t>CHIASSON</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>KENNEDY, MULLINS</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
           <t>WISE</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>MULLINS, CHIASSON</t>
-        </is>
-      </c>
-      <c r="E8" s="8" t="inlineStr">
-        <is>
-          <t>KENNEDY</t>
         </is>
       </c>
     </row>
@@ -1639,13 +1631,13 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>CHIASSON</t>
+          <t>WISE</t>
         </is>
       </c>
       <c r="D10" s="5" t="n"/>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>WISE</t>
+          <t>CHIASSON</t>
         </is>
       </c>
     </row>
@@ -1658,19 +1650,19 @@
       <c r="B11" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>KENNEDY</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>SAEED, CHIASSON</t>
+          <t>WISE, SAEED</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>WISE</t>
+          <t>CHIASSON</t>
         </is>
       </c>
     </row>
@@ -1688,14 +1680,14 @@
           <t>SAEED</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>KENNEDY, CHIASSON</t>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>WISE, KENNEDY</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>WISE</t>
+          <t>CHIASSON</t>
         </is>
       </c>
     </row>
@@ -1710,17 +1702,17 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
+          <t>WISE</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>KENNEDY, SAEED</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
           <t>CHIASSON</t>
-        </is>
-      </c>
-      <c r="D13" s="8" t="inlineStr">
-        <is>
-          <t>KENNEDY, SAEED</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>WISE</t>
         </is>
       </c>
     </row>
@@ -1735,17 +1727,17 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
+          <t>KENNEDY</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
           <t>SAEED</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="E14" s="3" t="inlineStr">
         <is>
           <t>CHIASSON</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>WISE</t>
         </is>
       </c>
     </row>
@@ -1758,19 +1750,19 @@
       <c r="B15" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="C15" s="8" t="inlineStr">
-        <is>
-          <t>KENNEDY</t>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>SAEED</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>SAEED, CHIASSON</t>
+          <t>WISE, KENNEDY</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>WISE</t>
+          <t>CHIASSON</t>
         </is>
       </c>
     </row>
@@ -1785,13 +1777,13 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>CHIASSON</t>
+          <t>WISE</t>
         </is>
       </c>
       <c r="D16" s="4" t="n"/>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>CHIASSON  (24H)</t>
+          <t>WISE  (24H)</t>
         </is>
       </c>
     </row>
@@ -1804,15 +1796,15 @@
       <c r="B17" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="C17" s="8" t="inlineStr">
-        <is>
-          <t>KENNEDY</t>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>CHIASSON</t>
         </is>
       </c>
       <c r="D17" s="5" t="n"/>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>SAEED</t>
+          <t>KENNEDY</t>
         </is>
       </c>
     </row>
@@ -1827,17 +1819,17 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>WISE</t>
-        </is>
-      </c>
-      <c r="D18" s="8" t="inlineStr">
-        <is>
-          <t>KENNEDY, VIVEKANANDAN</t>
+          <t>SAEED</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>WISE, VIVEKANANDAN</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>SAEED</t>
+          <t>KENNEDY</t>
         </is>
       </c>
     </row>
@@ -1855,14 +1847,14 @@
           <t>VIVEKANANDAN</t>
         </is>
       </c>
-      <c r="D19" s="8" t="inlineStr">
-        <is>
-          <t>WISE, KENNEDY</t>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>WISE, SAEED</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>SAEED</t>
+          <t>KENNEDY</t>
         </is>
       </c>
     </row>
@@ -1875,19 +1867,19 @@
       <c r="B20" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="C20" s="8" t="inlineStr">
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>WISE</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>SAEED, VIVEKANANDAN</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
         <is>
           <t>KENNEDY</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>WISE, VIVEKANANDAN</t>
-        </is>
-      </c>
-      <c r="E20" s="3" t="inlineStr">
-        <is>
-          <t>SAEED</t>
         </is>
       </c>
     </row>
@@ -1902,7 +1894,7 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>WISE</t>
+          <t>SAEED</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
@@ -1912,7 +1904,7 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>SAEED</t>
+          <t>KENNEDY</t>
         </is>
       </c>
     </row>
@@ -1930,14 +1922,14 @@
           <t>VIVEKANANDAN</t>
         </is>
       </c>
-      <c r="D22" s="8" t="inlineStr">
-        <is>
-          <t>WISE, KENNEDY</t>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>WISE, SAEED</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>SAEED</t>
+          <t>KENNEDY</t>
         </is>
       </c>
     </row>
@@ -1952,13 +1944,13 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>WISE</t>
+          <t>SAEED</t>
         </is>
       </c>
       <c r="D23" s="4" t="n"/>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>WISE  (24H)</t>
+          <t>SAEED  (24H)</t>
         </is>
       </c>
     </row>
@@ -1973,7 +1965,7 @@
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>SAEED</t>
+          <t>KENNEDY</t>
         </is>
       </c>
       <c r="D24" s="5" t="n"/>
@@ -1992,14 +1984,14 @@
       <c r="B25" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="C25" s="8" t="inlineStr">
-        <is>
-          <t>KENNEDY</t>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>WISE</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>WISE, SHETTY</t>
+          <t>KENNEDY, SHETTY</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
@@ -2022,7 +2014,7 @@
           <t>SHETTY</t>
         </is>
       </c>
-      <c r="D26" s="8" t="inlineStr">
+      <c r="D26" s="3" t="inlineStr">
         <is>
           <t>WISE, KENNEDY</t>
         </is>
@@ -2044,12 +2036,12 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>WISE</t>
-        </is>
-      </c>
-      <c r="D27" s="8" t="inlineStr">
-        <is>
-          <t>KENNEDY, SHETTY</t>
+          <t>KENNEDY</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>WISE, SHETTY</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
@@ -2069,12 +2061,12 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
+          <t>WISE</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
           <t>SHETTY</t>
-        </is>
-      </c>
-      <c r="D28" s="3" t="inlineStr">
-        <is>
-          <t>WISE</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
@@ -2094,12 +2086,12 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>WISE</t>
-        </is>
-      </c>
-      <c r="D29" s="8" t="inlineStr">
-        <is>
-          <t>KENNEDY, SHETTY</t>
+          <t>SHETTY</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>WISE, KENNEDY</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
@@ -2117,13 +2109,13 @@
       <c r="B30" s="4" t="n">
         <v>28</v>
       </c>
-      <c r="C30" s="8" t="inlineStr">
+      <c r="C30" s="4" t="inlineStr">
         <is>
           <t>KENNEDY</t>
         </is>
       </c>
       <c r="D30" s="4" t="n"/>
-      <c r="E30" s="8" t="inlineStr">
+      <c r="E30" s="4" t="inlineStr">
         <is>
           <t>KENNEDY  (24H)</t>
         </is>
@@ -2164,7 +2156,7 @@
           <t>WISE</t>
         </is>
       </c>
-      <c r="D32" s="8" t="inlineStr">
+      <c r="D32" s="3" t="inlineStr">
         <is>
           <t>KENNEDY, VIVEKANANDAN</t>
         </is>
@@ -5171,7 +5163,7 @@
           <t>MATSUOKA</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>KENNEDY, SHETTY</t>
         </is>
@@ -5191,7 +5183,7 @@
       <c r="B4" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>KENNEDY</t>
         </is>
@@ -5221,7 +5213,7 @@
           <t>SHETTY</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>KENNEDY, MATSUOKA</t>
         </is>
@@ -5241,7 +5233,7 @@
       <c r="B6" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>KENNEDY</t>
         </is>
@@ -5271,7 +5263,7 @@
           <t>MATSUOKA</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>KENNEDY, SHETTY</t>
         </is>
@@ -5318,7 +5310,7 @@
         </is>
       </c>
       <c r="D9" s="5" t="n"/>
-      <c r="E9" s="8" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>KENNEDY</t>
         </is>
@@ -5343,7 +5335,7 @@
           <t>SHETTY, PATEL</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>KENNEDY</t>
         </is>
@@ -5368,7 +5360,7 @@
           <t>MATSUOKA, SHETTY</t>
         </is>
       </c>
-      <c r="E11" s="8" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>KENNEDY</t>
         </is>
@@ -5393,7 +5385,7 @@
           <t>MATSUOKA, PATEL</t>
         </is>
       </c>
-      <c r="E12" s="8" t="inlineStr">
+      <c r="E12" s="3" t="inlineStr">
         <is>
           <t>KENNEDY</t>
         </is>
@@ -5418,7 +5410,7 @@
           <t>SHETTY</t>
         </is>
       </c>
-      <c r="E13" s="8" t="inlineStr">
+      <c r="E13" s="3" t="inlineStr">
         <is>
           <t>KENNEDY</t>
         </is>
@@ -5443,7 +5435,7 @@
           <t>SHETTY, PATEL</t>
         </is>
       </c>
-      <c r="E14" s="8" t="inlineStr">
+      <c r="E14" s="3" t="inlineStr">
         <is>
           <t>KENNEDY</t>
         </is>
@@ -5500,7 +5492,7 @@
       <c r="B17" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="C17" s="8" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>KENNEDY</t>
         </is>
@@ -5530,7 +5522,7 @@
           <t>BUTT</t>
         </is>
       </c>
-      <c r="D18" s="8" t="inlineStr">
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>KENNEDY, PATEL</t>
         </is>
@@ -5555,7 +5547,7 @@
           <t>PATEL</t>
         </is>
       </c>
-      <c r="D19" s="8" t="inlineStr">
+      <c r="D19" s="3" t="inlineStr">
         <is>
           <t>KENNEDY, BUTT</t>
         </is>
@@ -5605,7 +5597,7 @@
           <t>PATEL</t>
         </is>
       </c>
-      <c r="D21" s="8" t="inlineStr">
+      <c r="D21" s="3" t="inlineStr">
         <is>
           <t>KENNEDY, BUTT</t>
         </is>
@@ -5625,13 +5617,13 @@
       <c r="B22" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="C22" s="8" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>KENNEDY</t>
         </is>
       </c>
       <c r="D22" s="4" t="n"/>
-      <c r="E22" s="8" t="inlineStr">
+      <c r="E22" s="4" t="inlineStr">
         <is>
           <t>KENNEDY  (24H)</t>
         </is>
@@ -5672,7 +5664,7 @@
           <t>MATSUOKA</t>
         </is>
       </c>
-      <c r="D24" s="8" t="inlineStr">
+      <c r="D24" s="3" t="inlineStr">
         <is>
           <t>KENNEDY, ALMADHOOB</t>
         </is>
@@ -5697,7 +5689,7 @@
           <t>ALMADHOOB</t>
         </is>
       </c>
-      <c r="D25" s="8" t="inlineStr">
+      <c r="D25" s="3" t="inlineStr">
         <is>
           <t>KENNEDY, MATSUOKA</t>
         </is>
@@ -5717,7 +5709,7 @@
       <c r="B26" s="3" t="n">
         <v>24</v>
       </c>
-      <c r="C26" s="8" t="inlineStr">
+      <c r="C26" s="3" t="inlineStr">
         <is>
           <t>KENNEDY</t>
         </is>
@@ -5747,7 +5739,7 @@
           <t>ALMADHOOB</t>
         </is>
       </c>
-      <c r="D27" s="8" t="inlineStr">
+      <c r="D27" s="3" t="inlineStr">
         <is>
           <t>KENNEDY</t>
         </is>
@@ -5767,7 +5759,7 @@
       <c r="B28" s="3" t="n">
         <v>26</v>
       </c>
-      <c r="C28" s="8" t="inlineStr">
+      <c r="C28" s="3" t="inlineStr">
         <is>
           <t>KENNEDY</t>
         </is>
@@ -5834,7 +5826,7 @@
       <c r="B31" s="3" t="n">
         <v>29</v>
       </c>
-      <c r="C31" s="8" t="inlineStr">
+      <c r="C31" s="3" t="inlineStr">
         <is>
           <t>KENNEDY</t>
         </is>
@@ -5864,7 +5856,7 @@
           <t>RIVERA</t>
         </is>
       </c>
-      <c r="D32" s="8" t="inlineStr">
+      <c r="D32" s="3" t="inlineStr">
         <is>
           <t>KENNEDY, MATSUOKA</t>
         </is>
@@ -5889,7 +5881,7 @@
           <t>MATSUOKA</t>
         </is>
       </c>
-      <c r="D33" s="8" t="inlineStr">
+      <c r="D33" s="3" t="inlineStr">
         <is>
           <t>KENNEDY, RIVERA</t>
         </is>

</xml_diff>

<commit_message>
Accommodate Kennedy's Nov 7-8 weekend via a compliant slot swap
For Nov 1-13, Kennedy and the Lahey intern (Chiasson) swap slot roles: Kennedy
takes the Lahey slot (night float 11/1-6) and is fully OFF the 11/7-8 weekend;
Chiasson takes the LSH2 slot. This keeps every hard rule intact for those weeks
(Q4, one-LC/day, NF-consecutive, Saturday rules, days off). Kennedy keeps
Thanksgiving Day off and his single Saturday (11/28); he does one NF week and
one Saturday. Cost: one month-boundary coupling note (Fri 10/30 LC no longer
maps to the 11/1 NF, since Kennedy isn't present in October).

Fri 11/6 is his night-float shift (7:30pm on), so he's free until then; a full
Friday off is left off unless requested (it would ripple Q4).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J6EM8SxuZs5C898HeFBgt7
</commit_message>
<xml_diff>
--- a/intern_schedule_2026-2027/schedules/TYP_Intern_Schedule_Oct2026-Jun2027.xlsx
+++ b/intern_schedule_2026-2027/schedules/TYP_Intern_Schedule_Oct2026-Jun2027.xlsx
@@ -1474,7 +1474,7 @@
       <c r="D3" s="6" t="n"/>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>CHIASSON</t>
+          <t>KENNEDY</t>
         </is>
       </c>
     </row>
@@ -1494,12 +1494,12 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>KENNEDY, MULLINS</t>
+          <t>CHIASSON, MULLINS</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>CHIASSON</t>
+          <t>KENNEDY</t>
         </is>
       </c>
     </row>
@@ -1514,17 +1514,17 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
+          <t>CHIASSON</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>WISE, MULLINS</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
           <t>KENNEDY</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>WISE, MULLINS</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>CHIASSON</t>
         </is>
       </c>
     </row>
@@ -1544,12 +1544,12 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>WISE, KENNEDY</t>
+          <t>WISE, CHIASSON</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>CHIASSON</t>
+          <t>KENNEDY</t>
         </is>
       </c>
     </row>
@@ -1569,12 +1569,12 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
+          <t>CHIASSON</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
           <t>KENNEDY</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>CHIASSON</t>
         </is>
       </c>
     </row>
@@ -1589,17 +1589,17 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
+          <t>CHIASSON</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>WISE, MULLINS</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
           <t>KENNEDY</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>WISE, MULLINS</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>CHIASSON</t>
         </is>
       </c>
     </row>
@@ -1641,7 +1641,7 @@
       <c r="D10" s="6" t="n"/>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>KENNEDY</t>
+          <t>CHIASSON</t>
         </is>
       </c>
     </row>
@@ -1656,17 +1656,17 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
+          <t>KENNEDY</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>SAEED U, WISE</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
           <t>CHIASSON</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>SAEED U, WISE</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>KENNEDY</t>
         </is>
       </c>
     </row>
@@ -1686,12 +1686,12 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>CHIASSON, WISE</t>
+          <t>KENNEDY, WISE</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>KENNEDY</t>
+          <t>CHIASSON</t>
         </is>
       </c>
     </row>
@@ -1711,12 +1711,12 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>CHIASSON, SAEED U</t>
+          <t>KENNEDY, SAEED U</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>KENNEDY</t>
+          <t>CHIASSON</t>
         </is>
       </c>
     </row>
@@ -1731,17 +1731,17 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
+          <t>KENNEDY</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>SAEED U</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
           <t>CHIASSON</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>SAEED U</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>KENNEDY</t>
         </is>
       </c>
     </row>
@@ -1761,12 +1761,12 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>CHIASSON, WISE</t>
+          <t>KENNEDY, WISE</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>KENNEDY</t>
+          <t>CHIASSON</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add full-year audit document; revert to clean pure-march baseline
- Revert the November Kennedy slot swap so the committed schedule is the clean,
  fully-auditable pure-march baseline (November personal tweaks handled on the
  back end; re-enable via KEN_SWAP_DAYS in gen.py).
- Add generator/yearbook.py producing Intern_Schedule_FullYear.html: every month
  Oct 2026-Jun 2027 in one scrollable document plus a per-intern summary
  (NF nights, Saturdays, long/short call, days off, max consecutive days) and a
  compliance snapshot.
- Regenerate workbooks and RULES_COMPLIANCE.md for the baseline.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J6EM8SxuZs5C898HeFBgt7
</commit_message>
<xml_diff>
--- a/intern_schedule_2026-2027/schedules/TYP_Intern_Schedule_Oct2026-Jun2027.xlsx
+++ b/intern_schedule_2026-2027/schedules/TYP_Intern_Schedule_Oct2026-Jun2027.xlsx
@@ -1474,7 +1474,7 @@
       <c r="D3" s="6" t="n"/>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>KENNEDY</t>
+          <t>CHIASSON</t>
         </is>
       </c>
     </row>
@@ -1494,12 +1494,12 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>CHIASSON, MULLINS</t>
+          <t>KENNEDY, MULLINS</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>KENNEDY</t>
+          <t>CHIASSON</t>
         </is>
       </c>
     </row>
@@ -1514,17 +1514,17 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
+          <t>KENNEDY</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>WISE, MULLINS</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
           <t>CHIASSON</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>WISE, MULLINS</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>KENNEDY</t>
         </is>
       </c>
     </row>
@@ -1544,12 +1544,12 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>WISE, CHIASSON</t>
+          <t>WISE, KENNEDY</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>KENNEDY</t>
+          <t>CHIASSON</t>
         </is>
       </c>
     </row>
@@ -1569,12 +1569,12 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
+          <t>KENNEDY</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
           <t>CHIASSON</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>KENNEDY</t>
         </is>
       </c>
     </row>
@@ -1589,17 +1589,17 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
+          <t>KENNEDY</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>WISE, MULLINS</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
           <t>CHIASSON</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>WISE, MULLINS</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>KENNEDY</t>
         </is>
       </c>
     </row>
@@ -1641,7 +1641,7 @@
       <c r="D10" s="6" t="n"/>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>CHIASSON</t>
+          <t>KENNEDY</t>
         </is>
       </c>
     </row>
@@ -1656,17 +1656,17 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
+          <t>CHIASSON</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>SAEED U, WISE</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
           <t>KENNEDY</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>SAEED U, WISE</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>CHIASSON</t>
         </is>
       </c>
     </row>
@@ -1686,12 +1686,12 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>KENNEDY, WISE</t>
+          <t>CHIASSON, WISE</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>CHIASSON</t>
+          <t>KENNEDY</t>
         </is>
       </c>
     </row>
@@ -1711,12 +1711,12 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>KENNEDY, SAEED U</t>
+          <t>CHIASSON, SAEED U</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>CHIASSON</t>
+          <t>KENNEDY</t>
         </is>
       </c>
     </row>
@@ -1731,17 +1731,17 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
+          <t>CHIASSON</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>SAEED U</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
           <t>KENNEDY</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>SAEED U</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>CHIASSON</t>
         </is>
       </c>
     </row>
@@ -1761,12 +1761,12 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>KENNEDY, WISE</t>
+          <t>CHIASSON, WISE</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>CHIASSON</t>
+          <t>KENNEDY</t>
         </is>
       </c>
     </row>

</xml_diff>